<commit_message>
Exclude unavailable lipids and clean up formulation code repetition
</commit_message>
<xml_diff>
--- a/data/excel/Lipid properties.xlsx
+++ b/data/excel/Lipid properties.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hioa365-my.sharepoint.com/personal/masun1863_oslomet_no/Documents/Dokumenter/ML Feature Properties/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="321" documentId="8_{367B635D-84EA-430C-AF42-7ED26ADF74FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C235D68-C457-45F3-841A-1910A00A884C}"/>
+  <xr:revisionPtr revIDLastSave="326" documentId="8_{367B635D-84EA-430C-AF42-7ED26ADF74FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{832E1A18-B5BA-487D-9901-DE3EDFA1CA15}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{52E4DE00-B8E2-4867-A8EE-FA1EE720E88B}"/>
+    <workbookView xWindow="14130" yWindow="-16350" windowWidth="29040" windowHeight="15720" xr2:uid="{52E4DE00-B8E2-4867-A8EE-FA1EE720E88B}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="45">
   <si>
     <t>Hydrogen bond donor count</t>
   </si>
@@ -168,6 +168,9 @@
   </si>
   <si>
     <t>Is anionic</t>
+  </si>
+  <si>
+    <t>Information was collected from PubChem database of lipids, but formula weights were collected from Avanti Lipid site if the weights differed (DOTAP)</t>
   </si>
 </sst>
 </file>
@@ -184,7 +187,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -603,7 +605,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23386EA2-7693-4D8A-BE8A-2E3E5D43DF0D}">
-  <dimension ref="A1:S12"/>
+  <dimension ref="A1:S16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.1796875" bestFit="1" customWidth="1"/>
@@ -1108,7 +1110,7 @@
         <v>34</v>
       </c>
       <c r="D9">
-        <v>663.1</v>
+        <v>698.5</v>
       </c>
       <c r="E9">
         <v>37</v>
@@ -1202,7 +1204,7 @@
       <c r="O10" s="5">
         <v>1</v>
       </c>
-      <c r="P10">
+      <c r="P10" s="5">
         <v>1</v>
       </c>
       <c r="Q10" s="5">
@@ -1261,7 +1263,7 @@
       <c r="O11" s="5">
         <v>1</v>
       </c>
-      <c r="P11">
+      <c r="P11" s="5">
         <v>1</v>
       </c>
       <c r="Q11" s="5">
@@ -1331,6 +1333,11 @@
       </c>
       <c r="S12">
         <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -1347,15 +1354,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100014AE37F2444474EA4D68E839ECCDDD3" ma:contentTypeVersion="10" ma:contentTypeDescription="Opprett et nytt dokument." ma:contentTypeScope="" ma:versionID="264f9428646d58ecbe2ecf52a3651c39">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="b4431929-4c33-46cd-93fc-96c7645c6ebe" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1935da1053663dbc7bdeb9684e1c7118" ns3:_="">
     <xsd:import namespace="b4431929-4c33-46cd-93fc-96c7645c6ebe"/>
@@ -1537,6 +1535,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69D1889B-9597-4DC1-A6DD-7013C54D4562}">
   <ds:schemaRefs>
@@ -1554,14 +1561,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9E1EB5A0-0F25-45C1-BF1C-C4B740B60E41}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{89988FEA-A84F-4B0D-A80E-275F13FBDA1C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1579,6 +1578,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9E1EB5A0-0F25-45C1-BF1C-C4B740B60E41}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{fec81f12-6286-4550-8911-f446fcdafa1f}" enabled="0" method="" siteId="{fec81f12-6286-4550-8911-f446fcdafa1f}" removed="1"/>

</xml_diff>